<commit_message>
Versión 0.6.6 por verificar adicion de condicion.
</commit_message>
<xml_diff>
--- a/uploads/Enpoint_antivirus.xlsx
+++ b/uploads/Enpoint_antivirus.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9d4cd0066026126/Documentos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9d4cd0066026126/Documentos/Pruebas inventario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{9C6C54E5-0361-46F9-A8CF-515DC3E8DA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74F87471-27A2-4890-AFD7-5E3D97A226B2}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{9C6C54E5-0361-46F9-A8CF-515DC3E8DA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0AFC35C-8091-423C-81E8-A82A9D3894D1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{78BF6EA5-79BC-4845-B95A-4AA1573D2BC4}"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="15375" windowHeight="7875" xr2:uid="{78BF6EA5-79BC-4845-B95A-4AA1573D2BC4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Antivirus" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -163,6 +163,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>